<commit_message>
Quellenangabe und Hinweis auf geschlossene Geburtsabteilungen hinzugefügt
</commit_message>
<xml_diff>
--- a/Spitalliste_bereinigt_fuer_Dashboard.xlsx
+++ b/Spitalliste_bereinigt_fuer_Dashboard.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Marina Frei\Documents\Studium\Bachelorarbeit\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{118CF0FD-675B-45F5-BD6E-8F58F391388C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B6B212E-406C-4B44-A1BE-3714A42D4907}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -92,9 +92,6 @@
     <t>9.686234727259531</t>
   </si>
   <si>
-    <t>Spital Thusis</t>
-  </si>
-  <si>
     <t>Nein</t>
   </si>
   <si>
@@ -104,9 +101,6 @@
     <t>10.303826533438096</t>
   </si>
   <si>
-    <t>Centro sanitario Valposchiavo</t>
-  </si>
-  <si>
     <t>46.32304714423666</t>
   </si>
   <si>
@@ -168,6 +162,12 @@
   </si>
   <si>
     <t xml:space="preserve">Nein </t>
+  </si>
+  <si>
+    <t>Spital Thusis (Geburtsabteilung geschlossen)</t>
+  </si>
+  <si>
+    <t>Centro sanitario Valposchiavo (Geburtsabteilung geschlossen)</t>
   </si>
 </sst>
 </file>
@@ -585,10 +585,10 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B2" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>5</v>
@@ -602,10 +602,10 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B3" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>8</v>
@@ -619,10 +619,10 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B4" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>10</v>
@@ -636,7 +636,7 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B5" t="s">
         <v>12</v>
@@ -653,7 +653,7 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B6" t="s">
         <v>15</v>
@@ -670,16 +670,16 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B7" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C7" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D7" s="3" t="s">
         <v>20</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>21</v>
       </c>
       <c r="E7" t="s">
         <v>7</v>
@@ -687,16 +687,16 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B8" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="E8" t="s">
         <v>7</v>
@@ -704,36 +704,36 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B9" t="s">
+        <v>42</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="E9" t="s">
         <v>18</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="E9" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B10" t="s">
+        <v>43</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="D10" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="C10" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="D10" s="3" t="s">
-        <v>24</v>
-      </c>
       <c r="E10" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.35">

</xml_diff>